<commit_message>
Implementa algoritmo genetico con crossover ciclico, torneo, mutacion por intercambio y elitismo
</commit_message>
<xml_diff>
--- a/TablaCapitales_completa.xlsx
+++ b/TablaCapitales_completa.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="26">
   <si>
     <t>Distancias en kilómetros</t>
   </si>
   <si>
-    <t>Cdad. de Bs. As.</t>
+    <t>CABA</t>
   </si>
   <si>
     <t>Córdoba</t>
@@ -49,19 +49,19 @@
     <t>Rawson</t>
   </si>
   <si>
-    <t>Resisten- cia</t>
+    <t>Resistencia</t>
   </si>
   <si>
     <t>Río Gallegos</t>
   </si>
   <si>
-    <t>S.F.d.V.d. Catamarca</t>
-  </si>
-  <si>
-    <t>S.M. de Tucumán</t>
-  </si>
-  <si>
-    <t>S.S. de Jujuy</t>
+    <t>San Fernando del Valle de Catamarca</t>
+  </si>
+  <si>
+    <t>San Miguel de Tucumán</t>
+  </si>
+  <si>
+    <t>San Salvador de Jujuy</t>
   </si>
   <si>
     <t>Salta</t>
@@ -79,31 +79,13 @@
     <t>Santa Rosa</t>
   </si>
   <si>
-    <t>Sgo. Del Estero</t>
+    <t>Santiago del Estero</t>
   </si>
   <si>
     <t>Ushuaia</t>
   </si>
   <si>
     <t>Viedma</t>
-  </si>
-  <si>
-    <t>CABA</t>
-  </si>
-  <si>
-    <t>Resistencia</t>
-  </si>
-  <si>
-    <t>San Fernando del Valle de Catamarca</t>
-  </si>
-  <si>
-    <t>San Miguel de Tucumán</t>
-  </si>
-  <si>
-    <t>San Salvador de Jujuy</t>
-  </si>
-  <si>
-    <t>Santiago del Estero</t>
   </si>
   <si>
     <t>Elaboración propia - Las distancias son en línea recta y han sido calculadas con la utilización de un programa de conversión y transformación de coordenadas.</t>
@@ -206,6 +188,9 @@
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
+    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" vertical="top"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
@@ -213,9 +198,6 @@
       <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -469,79 +451,79 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="W1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="X1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="4" t="s">
+      <c r="Y1" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>25</v>
+      <c r="A2" s="2" t="s">
+        <v>1</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="7">
@@ -1366,7 +1348,7 @@
     </row>
     <row r="13">
       <c r="A13" s="9" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="B13" s="7">
         <v>794.0</v>
@@ -1516,7 +1498,7 @@
     </row>
     <row r="15">
       <c r="A15" s="9" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="B15" s="7">
         <v>979.0</v>
@@ -1591,7 +1573,7 @@
     </row>
     <row r="16">
       <c r="A16" s="9" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="B16" s="7">
         <v>1080.0</v>
@@ -1666,7 +1648,7 @@
     </row>
     <row r="17">
       <c r="A17" s="9" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="B17" s="7">
         <v>1334.0</v>
@@ -2116,7 +2098,7 @@
     </row>
     <row r="23">
       <c r="A23" s="9" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B23" s="7">
         <v>939.0</v>
@@ -2368,7 +2350,7 @@
     </row>
     <row r="27">
       <c r="A27" s="13" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="M27" s="12"/>
       <c r="N27" s="12"/>

</xml_diff>